<commit_message>
before completely removing the observer
</commit_message>
<xml_diff>
--- a/data/single_run/input/components/AXPs/axp_meisner.xlsx
+++ b/data/single_run/input/components/AXPs/axp_meisner.xlsx
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>r1_1,r1_2,r1_3,r1_4,r1_5</t>
+          <t>r1_1,r1_2,r1_3</t>
         </is>
       </c>
     </row>
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>r1_6,r1_7,r1_8,r1_9,r1_10</t>
+          <t>r1_4,r1_5,r1_6</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>r1_11,r1_12,r1_13,r1_14,r1_15</t>
+          <t>r1_7,r1_8,r1_9</t>
         </is>
       </c>
     </row>

</xml_diff>